<commit_message>
Create Input for adjusting transportation cost
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2107AD52-935C-455E-BFEF-C8804DF17A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,49 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="12">
+  <si>
+    <t>Commodity</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>costs_new</t>
+  </si>
+  <si>
+    <t>Methane</t>
+  </si>
+  <si>
+    <t>RU</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>LV</t>
+  </si>
+  <si>
+    <t>UA</t>
+  </si>
+  <si>
+    <t>BY</t>
+  </si>
+  <si>
+    <t>FI</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -66,6 +113,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}" name="Table1" displayName="Table1" ref="A1:D7" totalsRowShown="0">
+  <autoFilter ref="A1:D7" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{93EDB941-B8F5-4996-9581-769F7139396D}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{21C399AB-D53D-4749-81B3-2A84DB7771D3}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{6FCBAB15-DADA-433C-82F1-DE82DDCF62E4}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{759E5B24-8E0C-4B1A-9C8B-8E5872E855D2}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +390,118 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>99999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>99999999</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update data_prep to use existing df instead of importing an additional excel
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2107AD52-935C-455E-BFEF-C8804DF17A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0E6164-B09A-4ACD-B129-2FBDD9A331A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ark1" sheetId="1" r:id="rId1"/>
+    <sheet name="2021" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="25">
   <si>
     <t>Commodity</t>
   </si>
@@ -61,6 +61,45 @@
   </si>
   <si>
     <t>TR</t>
+  </si>
+  <si>
+    <t>RU_LNG_exp</t>
+  </si>
+  <si>
+    <t>IT_LNG_imp</t>
+  </si>
+  <si>
+    <t>BE_LNG_imp</t>
+  </si>
+  <si>
+    <t>FR_LNG_imp</t>
+  </si>
+  <si>
+    <t>EL_LNG_imp</t>
+  </si>
+  <si>
+    <t>HR_LNG_imp</t>
+  </si>
+  <si>
+    <t>LT_LNG_imp</t>
+  </si>
+  <si>
+    <t>NL_LNG_imp</t>
+  </si>
+  <si>
+    <t>PL_LNG_imp</t>
+  </si>
+  <si>
+    <t>PT_LNG_imp</t>
+  </si>
+  <si>
+    <t>ES_LNG_imp</t>
+  </si>
+  <si>
+    <t>TR_LNG_imp</t>
+  </si>
+  <si>
+    <t>UK_LNG_imp</t>
   </si>
 </sst>
 </file>
@@ -116,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}" name="Table1" displayName="Table1" ref="A1:D7" totalsRowShown="0">
-  <autoFilter ref="A1:D7" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}" name="Table1" displayName="Table1" ref="A1:D19" totalsRowShown="0">
+  <autoFilter ref="A1:D19" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{93EDB941-B8F5-4996-9581-769F7139396D}" name="Commodity"/>
     <tableColumn id="2" xr3:uid="{21C399AB-D53D-4749-81B3-2A84DB7771D3}" name="Source"/>
@@ -391,16 +430,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -414,7 +453,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -425,10 +464,10 @@
         <v>6</v>
       </c>
       <c r="D2">
-        <v>99999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -439,10 +478,10 @@
         <v>7</v>
       </c>
       <c r="D3">
-        <v>99999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -453,10 +492,10 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>99999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -467,10 +506,10 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>99999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -481,10 +520,10 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>99999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -495,7 +534,175 @@
         <v>11</v>
       </c>
       <c r="D7">
-        <v>99999999</v>
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add further scenario inputs and results
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -1,32 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DD4AD0-91A6-4ABE-986A-3CBB5E068F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE83F62C-FA79-467D-892F-85D1CCC4BEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
-    <sheet name="2024" sheetId="2" r:id="rId2"/>
+    <sheet name="2020_InvesPipes" sheetId="5" r:id="rId2"/>
+    <sheet name="2024" sheetId="2" r:id="rId3"/>
+    <sheet name="2024_USA" sheetId="3" r:id="rId4"/>
+    <sheet name="2024_QA" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="84">
   <si>
     <t>Commodity</t>
   </si>
@@ -116,6 +130,168 @@
   </si>
   <si>
     <t>LV_LNG_imp</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>HU</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>BE</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>LU</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>UK</t>
+  </si>
+  <si>
+    <t>BG</t>
+  </si>
+  <si>
+    <t>EL</t>
+  </si>
+  <si>
+    <t>MK</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>CZ</t>
+  </si>
+  <si>
+    <t>DK</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t>DZ</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>EE</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>LY</t>
+  </si>
+  <si>
+    <t>MD</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>limit_new</t>
+  </si>
+  <si>
+    <t>USA_LNG</t>
+  </si>
+  <si>
+    <t>BE_LNG</t>
+  </si>
+  <si>
+    <t>FR_LNG</t>
+  </si>
+  <si>
+    <t>EL_LNG</t>
+  </si>
+  <si>
+    <t>IT_LNG</t>
+  </si>
+  <si>
+    <t>HR_LNG</t>
+  </si>
+  <si>
+    <t>LT_LNG</t>
+  </si>
+  <si>
+    <t>NL_LNG</t>
+  </si>
+  <si>
+    <t>PL_LNG</t>
+  </si>
+  <si>
+    <t>PT_LNG</t>
+  </si>
+  <si>
+    <t>ES_LNG</t>
+  </si>
+  <si>
+    <t>TR_LNG</t>
+  </si>
+  <si>
+    <t>UK_LNG</t>
+  </si>
+  <si>
+    <t>EE_LNG</t>
+  </si>
+  <si>
+    <t>FI_LNG</t>
+  </si>
+  <si>
+    <t>DE_LNG</t>
+  </si>
+  <si>
+    <t>IE_LNG</t>
+  </si>
+  <si>
+    <t>LV_LNG</t>
+  </si>
+  <si>
+    <t>QA_LNG</t>
   </si>
 </sst>
 </file>
@@ -191,6 +367,32 @@
     <tableColumn id="2" xr3:uid="{103C14AE-57A4-42EA-823B-79D14F8CB715}" name="Source"/>
     <tableColumn id="3" xr3:uid="{D5299053-FF13-4455-BBF3-EE8EB2D74756}" name="Destination"/>
     <tableColumn id="4" xr3:uid="{C72F0041-07FB-4B7B-B051-24184E510B45}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}" name="Table4" displayName="Table4" ref="A1:D41" totalsRowShown="0">
+  <autoFilter ref="A1:D41" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0A947DEB-26EB-4BD6-9532-5DD97ED5CC13}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{D5A1A772-C72D-455C-BA11-F5A9F62EF252}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{0605D032-B1CF-48E4-8D07-F67827D0B320}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{F5D77DD0-41BB-43C0-B518-B39EB35EF457}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}" name="Table3" displayName="Table3" ref="A1:D41" totalsRowShown="0">
+  <autoFilter ref="A1:D41" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{2645C0F2-1C87-4F7A-BABA-338A3C3BBAFE}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{973842F3-D49E-44B5-BDB2-51FF787DAA0A}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{A42789D1-B2CE-46DE-AC55-0295057DFC4F}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{F6BF22FC-7CBE-4FB2-9ACF-135D18D14394}" name="costs_new"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -743,6 +945,1869 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23A2BBDA-BF95-4C19-8BF8-08ECCB4DC5E7}">
+  <dimension ref="A1:E109"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" t="s">
+        <v>38</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="E33">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>52</v>
+      </c>
+      <c r="C40" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" t="s">
+        <v>30</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
+        <v>53</v>
+      </c>
+      <c r="C45" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" t="s">
+        <v>57</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>4</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" t="s">
+        <v>37</v>
+      </c>
+      <c r="C48" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+      <c r="E48">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" t="s">
+        <v>37</v>
+      </c>
+      <c r="C50" t="s">
+        <v>53</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>4</v>
+      </c>
+      <c r="B51" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>4</v>
+      </c>
+      <c r="B52" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" t="s">
+        <v>34</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" t="s">
+        <v>58</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" t="s">
+        <v>45</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" t="s">
+        <v>35</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="E56">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>4</v>
+      </c>
+      <c r="B57" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57" t="s">
+        <v>32</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>4</v>
+      </c>
+      <c r="B58" t="s">
+        <v>31</v>
+      </c>
+      <c r="C58" t="s">
+        <v>48</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>4</v>
+      </c>
+      <c r="B59" t="s">
+        <v>31</v>
+      </c>
+      <c r="C59" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>4</v>
+      </c>
+      <c r="B60" t="s">
+        <v>46</v>
+      </c>
+      <c r="C60" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="E60">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>4</v>
+      </c>
+      <c r="B61" t="s">
+        <v>46</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>4</v>
+      </c>
+      <c r="B62" t="s">
+        <v>38</v>
+      </c>
+      <c r="C62" t="s">
+        <v>36</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>4</v>
+      </c>
+      <c r="B63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" t="s">
+        <v>56</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" t="s">
+        <v>46</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>4</v>
+      </c>
+      <c r="B65" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" t="s">
+        <v>59</v>
+      </c>
+      <c r="C66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="E66">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>4</v>
+      </c>
+      <c r="B67" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" t="s">
+        <v>53</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>4</v>
+      </c>
+      <c r="B68" t="s">
+        <v>60</v>
+      </c>
+      <c r="C68" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>4</v>
+      </c>
+      <c r="B69" t="s">
+        <v>60</v>
+      </c>
+      <c r="C69" t="s">
+        <v>8</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>4</v>
+      </c>
+      <c r="B70" t="s">
+        <v>39</v>
+      </c>
+      <c r="C70" t="s">
+        <v>36</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>4</v>
+      </c>
+      <c r="B71" t="s">
+        <v>39</v>
+      </c>
+      <c r="C71" t="s">
+        <v>6</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+      <c r="E71">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>4</v>
+      </c>
+      <c r="B72" t="s">
+        <v>39</v>
+      </c>
+      <c r="C72" t="s">
+        <v>40</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>4</v>
+      </c>
+      <c r="B73" t="s">
+        <v>61</v>
+      </c>
+      <c r="C73" t="s">
+        <v>36</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+      <c r="E73">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" t="s">
+        <v>61</v>
+      </c>
+      <c r="C74" t="s">
+        <v>6</v>
+      </c>
+      <c r="D74">
+        <v>1</v>
+      </c>
+      <c r="E74">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>4</v>
+      </c>
+      <c r="B75" t="s">
+        <v>61</v>
+      </c>
+      <c r="C75" t="s">
+        <v>37</v>
+      </c>
+      <c r="D75">
+        <v>1</v>
+      </c>
+      <c r="E75">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>4</v>
+      </c>
+      <c r="B76" t="s">
+        <v>61</v>
+      </c>
+      <c r="C76" t="s">
+        <v>39</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
+      </c>
+      <c r="E76">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" t="s">
+        <v>61</v>
+      </c>
+      <c r="C77" t="s">
+        <v>40</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>4</v>
+      </c>
+      <c r="B78" t="s">
+        <v>47</v>
+      </c>
+      <c r="C78" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78">
+        <v>1</v>
+      </c>
+      <c r="E78">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>4</v>
+      </c>
+      <c r="B79" t="s">
+        <v>57</v>
+      </c>
+      <c r="C79" t="s">
+        <v>53</v>
+      </c>
+      <c r="D79">
+        <v>1</v>
+      </c>
+      <c r="E79">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" t="s">
+        <v>44</v>
+      </c>
+      <c r="C80" t="s">
+        <v>41</v>
+      </c>
+      <c r="D80">
+        <v>1</v>
+      </c>
+      <c r="E80">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>4</v>
+      </c>
+      <c r="B81" t="s">
+        <v>44</v>
+      </c>
+      <c r="C81" t="s">
+        <v>33</v>
+      </c>
+      <c r="D81">
+        <v>1</v>
+      </c>
+      <c r="E81">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>4</v>
+      </c>
+      <c r="B82" t="s">
+        <v>44</v>
+      </c>
+      <c r="C82" t="s">
+        <v>60</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>4</v>
+      </c>
+      <c r="B83" t="s">
+        <v>44</v>
+      </c>
+      <c r="C83" t="s">
+        <v>8</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>4</v>
+      </c>
+      <c r="B84" t="s">
+        <v>45</v>
+      </c>
+      <c r="C84" t="s">
+        <v>62</v>
+      </c>
+      <c r="D84">
+        <v>1</v>
+      </c>
+      <c r="E84">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>4</v>
+      </c>
+      <c r="B85" t="s">
+        <v>45</v>
+      </c>
+      <c r="C85" t="s">
+        <v>41</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
+      </c>
+      <c r="E85">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>4</v>
+      </c>
+      <c r="B86" t="s">
+        <v>45</v>
+      </c>
+      <c r="C86" t="s">
+        <v>33</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>4</v>
+      </c>
+      <c r="B87" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" t="s">
+        <v>9</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>4</v>
+      </c>
+      <c r="B88" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" t="s">
+        <v>6</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>4</v>
+      </c>
+      <c r="B89" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" t="s">
+        <v>10</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
+      </c>
+      <c r="E89">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>4</v>
+      </c>
+      <c r="B90" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>4</v>
+      </c>
+      <c r="B91" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" t="s">
+        <v>11</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="E91">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>4</v>
+      </c>
+      <c r="B92" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" t="s">
+        <v>8</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>4</v>
+      </c>
+      <c r="B93" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" t="s">
+        <v>58</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>4</v>
+      </c>
+      <c r="B94" t="s">
+        <v>34</v>
+      </c>
+      <c r="C94" t="s">
+        <v>31</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>4</v>
+      </c>
+      <c r="B95" t="s">
+        <v>35</v>
+      </c>
+      <c r="C95" t="s">
+        <v>32</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>4</v>
+      </c>
+      <c r="B96" t="s">
+        <v>35</v>
+      </c>
+      <c r="C96" t="s">
+        <v>49</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>4</v>
+      </c>
+      <c r="B97" t="s">
+        <v>35</v>
+      </c>
+      <c r="C97" t="s">
+        <v>33</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>4</v>
+      </c>
+      <c r="B98" t="s">
+        <v>35</v>
+      </c>
+      <c r="C98" t="s">
+        <v>8</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>4</v>
+      </c>
+      <c r="B99" t="s">
+        <v>55</v>
+      </c>
+      <c r="C99" t="s">
+        <v>31</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>4</v>
+      </c>
+      <c r="B100" t="s">
+        <v>11</v>
+      </c>
+      <c r="C100" t="s">
+        <v>41</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>4</v>
+      </c>
+      <c r="B101" t="s">
+        <v>11</v>
+      </c>
+      <c r="C101" t="s">
+        <v>42</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>4</v>
+      </c>
+      <c r="B102" t="s">
+        <v>8</v>
+      </c>
+      <c r="C102" t="s">
+        <v>33</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>4</v>
+      </c>
+      <c r="B103" t="s">
+        <v>8</v>
+      </c>
+      <c r="C103" t="s">
+        <v>60</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>4</v>
+      </c>
+      <c r="B104" t="s">
+        <v>8</v>
+      </c>
+      <c r="C104" t="s">
+        <v>47</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
+      </c>
+      <c r="E104">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>4</v>
+      </c>
+      <c r="B105" t="s">
+        <v>8</v>
+      </c>
+      <c r="C105" t="s">
+        <v>44</v>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="E105">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>4</v>
+      </c>
+      <c r="B106" t="s">
+        <v>8</v>
+      </c>
+      <c r="C106" t="s">
+        <v>35</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>4</v>
+      </c>
+      <c r="B107" t="s">
+        <v>40</v>
+      </c>
+      <c r="C107" t="s">
+        <v>36</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="E107">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>4</v>
+      </c>
+      <c r="B108" t="s">
+        <v>40</v>
+      </c>
+      <c r="C108" t="s">
+        <v>63</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
+      </c>
+      <c r="E108">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>4</v>
+      </c>
+      <c r="B109" t="s">
+        <v>40</v>
+      </c>
+      <c r="C109" t="s">
+        <v>39</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
+      </c>
+      <c r="E109">
+        <v>1000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2388587D-5E96-496D-9D26-761102F3935F}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1095,4 +3160,1188 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8977CDA9-B827-4B14-B0EF-E8B18335E1FD}">
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41">
+        <v>999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E7BF925-CC6B-405E-A306-8078742D0F1F}">
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41">
+        <v>999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add data update for case variation Norway
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE83F62C-FA79-467D-892F-85D1CCC4BEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBBC52D-9F2E-4CC8-8E10-D81DCF332D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="2024" sheetId="2" r:id="rId3"/>
     <sheet name="2024_USA" sheetId="3" r:id="rId4"/>
     <sheet name="2024_QA" sheetId="4" r:id="rId5"/>
+    <sheet name="2024_NOR" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="85">
   <si>
     <t>Commodity</t>
   </si>
@@ -292,6 +293,9 @@
   </si>
   <si>
     <t>QA_LNG</t>
+  </si>
+  <si>
+    <t>capacity_new</t>
   </si>
 </sst>
 </file>
@@ -393,6 +397,20 @@
     <tableColumn id="2" xr3:uid="{973842F3-D49E-44B5-BDB2-51FF787DAA0A}" name="Source"/>
     <tableColumn id="3" xr3:uid="{A42789D1-B2CE-46DE-AC55-0295057DFC4F}" name="Destination"/>
     <tableColumn id="4" xr3:uid="{F6BF22FC-7CBE-4FB2-9ACF-135D18D14394}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{FEB0F6EA-E60A-4566-BA0E-BF2AF5C97F48}" name="Table136" displayName="Table136" ref="A1:E28" totalsRowShown="0">
+  <autoFilter ref="A1:E28" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{06B2EE92-59E8-4B5C-B2CD-0D0EE3B58016}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{57E5570B-C2AA-4B2B-8493-88F8C5CB97AA}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{9874643B-57D7-4868-B1C0-F355AB9952C9}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{D924A804-C9E2-43F5-9843-9C52BA9C4FAD}" name="costs_new"/>
+    <tableColumn id="5" xr3:uid="{D19A91CC-FB88-41CD-86FA-402CD4D7BEA4}" name="capacity_new"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4344,4 +4362,499 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C547CAD-73AE-429A-84D2-4495A6C1A811}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>999999</v>
+      </c>
+      <c r="E2">
+        <v>513190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>999999</v>
+      </c>
+      <c r="E3">
+        <v>61320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>999999</v>
+      </c>
+      <c r="E4">
+        <v>486910</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>999999</v>
+      </c>
+      <c r="E5">
+        <v>439277.49999999988</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>999999</v>
+      </c>
+      <c r="E6">
+        <v>80300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>999999</v>
+      </c>
+      <c r="E7">
+        <v>349998.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+      <c r="E8">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+      <c r="E9">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+      <c r="E10">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+      <c r="E11">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+      <c r="E12">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+      <c r="E13">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+      <c r="E14">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+      <c r="E15">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+      <c r="E16">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+      <c r="E17">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+      <c r="E18">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
+      </c>
+      <c r="E19">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20">
+        <v>999999</v>
+      </c>
+      <c r="E20">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21">
+        <v>999999</v>
+      </c>
+      <c r="E21">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22">
+        <v>999999</v>
+      </c>
+      <c r="E22">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23">
+        <v>999999</v>
+      </c>
+      <c r="E23">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24">
+        <v>999999</v>
+      </c>
+      <c r="E24">
+        <v>9999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25">
+        <v>2635.6088276270129</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>2452.8956460783979</v>
+      </c>
+      <c r="E26">
+        <v>234.48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27">
+        <v>3449.967874173466</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28">
+        <v>2312.4197737153231</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update data for Norway reduction case
some pipelines from Norway are not available
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F74932-87C5-4310-944A-B3A545CF3028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4AF19B-9AED-4482-990B-1220D46ED2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -2531,7 +2531,7 @@
         <v>999999</v>
       </c>
       <c r="E2">
-        <v>513190</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2548,7 +2548,7 @@
         <v>999999</v>
       </c>
       <c r="E3">
-        <v>61320</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -2565,7 +2565,7 @@
         <v>999999</v>
       </c>
       <c r="E4">
-        <v>486910</v>
+        <v>1992720.7302134999</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2582,7 +2582,7 @@
         <v>999999</v>
       </c>
       <c r="E5">
-        <v>439277.49999999988</v>
+        <v>439277.49999999994</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -2599,7 +2599,7 @@
         <v>999999</v>
       </c>
       <c r="E6">
-        <v>80300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -2939,7 +2939,7 @@
         <v>2452.8956460783979</v>
       </c>
       <c r="E26">
-        <v>234.48</v>
+        <v>205170</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
run 2035 scenario variations
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4AF19B-9AED-4482-990B-1220D46ED2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A52D2FD-6BB9-40ED-A375-38CC7BA226A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
     <sheet name="2024" sheetId="2" r:id="rId2"/>
-    <sheet name="2024_USA" sheetId="3" r:id="rId3"/>
-    <sheet name="2024_QA" sheetId="4" r:id="rId4"/>
-    <sheet name="2024_NOR" sheetId="6" r:id="rId5"/>
-    <sheet name="2024_InvesPipes" sheetId="5" r:id="rId6"/>
+    <sheet name="2035" sheetId="7" r:id="rId3"/>
+    <sheet name="2024_USA" sheetId="3" r:id="rId4"/>
+    <sheet name="2024_QA" sheetId="4" r:id="rId5"/>
+    <sheet name="2024_NOR" sheetId="6" r:id="rId6"/>
+    <sheet name="2024_InvesPipes" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="81">
   <si>
     <t>Commodity</t>
   </si>
@@ -365,6 +366,19 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2E4244DF-E5BF-4A0E-8F99-4EC8DA9D37A0}" name="Table137" displayName="Table137" ref="A1:D24" totalsRowShown="0">
+  <autoFilter ref="A1:D24" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{40657536-7F27-4026-B8F3-FD897B9ED76C}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{C13810D6-089B-46C8-BA66-B5F657F9865E}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{7C0D1425-23BD-44EA-8A5F-4F1C3BB6EFCB}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{B5E8E473-41FA-492B-821E-3D41A4D0D004}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}" name="Table4" displayName="Table4" ref="A1:D41" totalsRowShown="0">
   <autoFilter ref="A1:D41" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}"/>
   <tableColumns count="4">
@@ -377,7 +391,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}" name="Table3" displayName="Table3" ref="A1:D41" totalsRowShown="0">
   <autoFilter ref="A1:D41" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}"/>
   <tableColumns count="4">
@@ -390,7 +404,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{FEB0F6EA-E60A-4566-BA0E-BF2AF5C97F48}" name="Table136" displayName="Table136" ref="A1:E28" totalsRowShown="0">
   <autoFilter ref="A1:E28" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
   <tableColumns count="5">
@@ -1306,6 +1320,361 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{943B3CE1-E7F7-4C15-AD65-81C37CD6AF52}">
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24">
+        <v>999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8977CDA9-B827-4B14-B0EF-E8B18335E1FD}">
   <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1897,7 +2266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E7BF925-CC6B-405E-A306-8078742D0F1F}">
   <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2489,7 +2858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C547CAD-73AE-429A-84D2-4495A6C1A811}">
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2984,7 +3353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23A2BBDA-BF95-4C19-8BF8-08ECCB4DC5E7}">
   <dimension ref="A1:E104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
update investment cost scenario update date file
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A52D2FD-6BB9-40ED-A375-38CC7BA226A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB6F974-96A3-4932-924B-6DEF3822B94B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -3386,7 +3386,7 @@
         <v>31</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E2">
         <v>1000000</v>
@@ -3403,7 +3403,7 @@
         <v>33</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E3">
         <v>1000000</v>
@@ -3420,7 +3420,7 @@
         <v>35</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E4">
         <v>1000000</v>
@@ -3437,7 +3437,7 @@
         <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E5">
         <v>1000000</v>
@@ -3454,7 +3454,7 @@
         <v>34</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E6">
         <v>1000000</v>
@@ -3471,7 +3471,7 @@
         <v>31</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E7">
         <v>1000000</v>
@@ -3488,7 +3488,7 @@
         <v>6</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E8">
         <v>1000000</v>
@@ -3505,7 +3505,7 @@
         <v>40</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E9">
         <v>1000000</v>
@@ -3522,7 +3522,7 @@
         <v>39</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E10">
         <v>1000000</v>
@@ -3539,7 +3539,7 @@
         <v>38</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E11">
         <v>1000000</v>
@@ -3556,7 +3556,7 @@
         <v>37</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E12">
         <v>1000000</v>
@@ -3573,7 +3573,7 @@
         <v>44</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E13">
         <v>1000000</v>
@@ -3590,7 +3590,7 @@
         <v>45</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E14">
         <v>1000000</v>
@@ -3607,7 +3607,7 @@
         <v>11</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E15">
         <v>1000000</v>
@@ -3624,7 +3624,7 @@
         <v>42</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E16">
         <v>1000000</v>
@@ -3641,7 +3641,7 @@
         <v>43</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E17">
         <v>1000000</v>
@@ -3658,7 +3658,7 @@
         <v>47</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E18">
         <v>1000000</v>
@@ -3675,7 +3675,7 @@
         <v>8</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E19">
         <v>1000000</v>
@@ -3692,7 +3692,7 @@
         <v>46</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E20">
         <v>1000000</v>
@@ -3709,7 +3709,7 @@
         <v>6</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E21">
         <v>1000000</v>
@@ -3726,7 +3726,7 @@
         <v>31</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E22">
         <v>1000000</v>
@@ -3743,7 +3743,7 @@
         <v>37</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E23">
         <v>1000000</v>
@@ -3760,7 +3760,7 @@
         <v>47</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E24">
         <v>1000000</v>
@@ -3777,7 +3777,7 @@
         <v>35</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E25">
         <v>1000000</v>
@@ -3794,7 +3794,7 @@
         <v>6</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E26">
         <v>1000000</v>
@@ -3811,7 +3811,7 @@
         <v>32</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E27">
         <v>1000000</v>
@@ -3828,7 +3828,7 @@
         <v>38</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E28">
         <v>1000000</v>
@@ -3845,7 +3845,7 @@
         <v>37</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E29">
         <v>1000000</v>
@@ -3862,7 +3862,7 @@
         <v>50</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E30">
         <v>1000000</v>
@@ -3879,7 +3879,7 @@
         <v>48</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E31">
         <v>1000000</v>
@@ -3896,7 +3896,7 @@
         <v>49</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E32">
         <v>1000000</v>
@@ -3913,7 +3913,7 @@
         <v>47</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E33">
         <v>1000000</v>
@@ -3930,7 +3930,7 @@
         <v>36</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E34">
         <v>1000000</v>
@@ -3947,7 +3947,7 @@
         <v>39</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E35">
         <v>1000000</v>
@@ -3964,7 +3964,7 @@
         <v>6</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E36">
         <v>1000000</v>
@@ -3981,7 +3981,7 @@
         <v>51</v>
       </c>
       <c r="D37">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E37">
         <v>1000000</v>
@@ -3998,7 +3998,7 @@
         <v>47</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E38">
         <v>1000000</v>
@@ -4015,7 +4015,7 @@
         <v>7</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E39">
         <v>1000000</v>
@@ -4032,7 +4032,7 @@
         <v>10</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E40">
         <v>1000000</v>
@@ -4049,7 +4049,7 @@
         <v>41</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E41">
         <v>1000000</v>
@@ -4066,7 +4066,7 @@
         <v>30</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E42">
         <v>1000000</v>
@@ -4083,7 +4083,7 @@
         <v>37</v>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E43">
         <v>1000000</v>
@@ -4100,7 +4100,7 @@
         <v>54</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E44">
         <v>1000000</v>
@@ -4117,7 +4117,7 @@
         <v>53</v>
       </c>
       <c r="D45">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E45">
         <v>1000000</v>
@@ -4134,7 +4134,7 @@
         <v>6</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E46">
         <v>1000000</v>
@@ -4151,7 +4151,7 @@
         <v>36</v>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E47">
         <v>1000000</v>
@@ -4168,7 +4168,7 @@
         <v>52</v>
       </c>
       <c r="D48">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E48">
         <v>1000000</v>
@@ -4185,7 +4185,7 @@
         <v>48</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E49">
         <v>1000000</v>
@@ -4202,7 +4202,7 @@
         <v>34</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E50">
         <v>1000000</v>
@@ -4219,7 +4219,7 @@
         <v>33</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E51">
         <v>1000000</v>
@@ -4236,7 +4236,7 @@
         <v>55</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E52">
         <v>1000000</v>
@@ -4253,7 +4253,7 @@
         <v>35</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E53">
         <v>1000000</v>
@@ -4270,7 +4270,7 @@
         <v>44</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E54">
         <v>1000000</v>
@@ -4287,7 +4287,7 @@
         <v>45</v>
       </c>
       <c r="D55">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E55">
         <v>1000000</v>
@@ -4304,7 +4304,7 @@
         <v>32</v>
       </c>
       <c r="D56">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E56">
         <v>1000000</v>
@@ -4321,7 +4321,7 @@
         <v>48</v>
       </c>
       <c r="D57">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E57">
         <v>1000000</v>
@@ -4338,7 +4338,7 @@
         <v>34</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E58">
         <v>1000000</v>
@@ -4355,7 +4355,7 @@
         <v>7</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E59">
         <v>1000000</v>
@@ -4372,7 +4372,7 @@
         <v>5</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E60">
         <v>1000000</v>
@@ -4389,7 +4389,7 @@
         <v>47</v>
       </c>
       <c r="D61">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E61">
         <v>1000000</v>
@@ -4406,7 +4406,7 @@
         <v>36</v>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E62">
         <v>1000000</v>
@@ -4423,7 +4423,7 @@
         <v>53</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E63">
         <v>1000000</v>
@@ -4440,7 +4440,7 @@
         <v>46</v>
       </c>
       <c r="D64">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E64">
         <v>1000000</v>
@@ -4457,7 +4457,7 @@
         <v>5</v>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E65">
         <v>1000000</v>
@@ -4474,7 +4474,7 @@
         <v>44</v>
       </c>
       <c r="D66">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E66">
         <v>1000000</v>
@@ -4491,7 +4491,7 @@
         <v>8</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E67">
         <v>1000000</v>
@@ -4508,7 +4508,7 @@
         <v>40</v>
       </c>
       <c r="D68">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E68">
         <v>1000000</v>
@@ -4525,7 +4525,7 @@
         <v>36</v>
       </c>
       <c r="D69">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E69">
         <v>1000000</v>
@@ -4542,7 +4542,7 @@
         <v>6</v>
       </c>
       <c r="D70">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E70">
         <v>1000000</v>
@@ -4559,7 +4559,7 @@
         <v>6</v>
       </c>
       <c r="D71">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E71">
         <v>1000000</v>
@@ -4576,7 +4576,7 @@
         <v>39</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E72">
         <v>1000000</v>
@@ -4593,7 +4593,7 @@
         <v>40</v>
       </c>
       <c r="D73">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E73">
         <v>1000000</v>
@@ -4610,7 +4610,7 @@
         <v>37</v>
       </c>
       <c r="D74">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E74">
         <v>1000000</v>
@@ -4627,7 +4627,7 @@
         <v>50</v>
       </c>
       <c r="D75">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E75">
         <v>1000000</v>
@@ -4644,7 +4644,7 @@
         <v>36</v>
       </c>
       <c r="D76">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E76">
         <v>1000000</v>
@@ -4661,7 +4661,7 @@
         <v>35</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E77">
         <v>1000000</v>
@@ -4678,7 +4678,7 @@
         <v>6</v>
       </c>
       <c r="D78">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E78">
         <v>1000000</v>
@@ -4695,7 +4695,7 @@
         <v>50</v>
       </c>
       <c r="D79">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E79">
         <v>1000000</v>
@@ -4712,7 +4712,7 @@
         <v>52</v>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E80">
         <v>1000000</v>
@@ -4729,7 +4729,7 @@
         <v>33</v>
       </c>
       <c r="D81">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E81">
         <v>1000000</v>
@@ -4746,7 +4746,7 @@
         <v>56</v>
       </c>
       <c r="D82">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E82">
         <v>1000000</v>
@@ -4763,7 +4763,7 @@
         <v>41</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E83">
         <v>1000000</v>
@@ -4780,7 +4780,7 @@
         <v>8</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E84">
         <v>1000000</v>
@@ -4797,7 +4797,7 @@
         <v>58</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E85">
         <v>1000000</v>
@@ -4814,7 +4814,7 @@
         <v>33</v>
       </c>
       <c r="D86">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E86">
         <v>1000000</v>
@@ -4831,7 +4831,7 @@
         <v>41</v>
       </c>
       <c r="D87">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E87">
         <v>1000000</v>
@@ -4848,7 +4848,7 @@
         <v>55</v>
       </c>
       <c r="D88">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E88">
         <v>1000000</v>
@@ -4865,7 +4865,7 @@
         <v>31</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E89">
         <v>1000000</v>
@@ -4882,7 +4882,7 @@
         <v>32</v>
       </c>
       <c r="D90">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E90">
         <v>1000000</v>
@@ -4899,7 +4899,7 @@
         <v>49</v>
       </c>
       <c r="D91">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E91">
         <v>1000000</v>
@@ -4916,7 +4916,7 @@
         <v>47</v>
       </c>
       <c r="D92">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E92">
         <v>1000000</v>
@@ -4933,7 +4933,7 @@
         <v>33</v>
       </c>
       <c r="D93">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E93">
         <v>1000000</v>
@@ -4950,7 +4950,7 @@
         <v>8</v>
       </c>
       <c r="D94">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E94">
         <v>1000000</v>
@@ -4967,7 +4967,7 @@
         <v>41</v>
       </c>
       <c r="D95">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E95">
         <v>1000000</v>
@@ -4984,7 +4984,7 @@
         <v>42</v>
       </c>
       <c r="D96">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E96">
         <v>1000000</v>
@@ -5001,7 +5001,7 @@
         <v>47</v>
       </c>
       <c r="D97">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E97">
         <v>1000000</v>
@@ -5018,7 +5018,7 @@
         <v>33</v>
       </c>
       <c r="D98">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E98">
         <v>1000000</v>
@@ -5035,7 +5035,7 @@
         <v>35</v>
       </c>
       <c r="D99">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E99">
         <v>1000000</v>
@@ -5052,7 +5052,7 @@
         <v>56</v>
       </c>
       <c r="D100">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E100">
         <v>1000000</v>
@@ -5069,7 +5069,7 @@
         <v>44</v>
       </c>
       <c r="D101">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E101">
         <v>1000000</v>
@@ -5086,7 +5086,7 @@
         <v>59</v>
       </c>
       <c r="D102">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E102">
         <v>1000000</v>
@@ -5103,7 +5103,7 @@
         <v>36</v>
       </c>
       <c r="D103">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E103">
         <v>1000000</v>
@@ -5120,7 +5120,7 @@
         <v>39</v>
       </c>
       <c r="D104">
-        <v>1</v>
+        <v>0.50735667174023336</v>
       </c>
       <c r="E104">
         <v>1000000</v>

</xml_diff>

<commit_message>
add Norwegian LNG connections for NO pipe interruption case
and bug fix that the scenario update files contain _exp and _imp suffix for all connections.
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB6F974-96A3-4932-924B-6DEF3822B94B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE41426D-03F5-4EC5-93E5-396CA3AA20BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="64">
   <si>
     <t>Commodity</t>
   </si>
@@ -227,64 +227,13 @@
     <t>limit_new</t>
   </si>
   <si>
-    <t>USA_LNG</t>
-  </si>
-  <si>
-    <t>BE_LNG</t>
-  </si>
-  <si>
-    <t>FR_LNG</t>
-  </si>
-  <si>
-    <t>EL_LNG</t>
-  </si>
-  <si>
-    <t>IT_LNG</t>
-  </si>
-  <si>
-    <t>HR_LNG</t>
-  </si>
-  <si>
-    <t>LT_LNG</t>
-  </si>
-  <si>
-    <t>NL_LNG</t>
-  </si>
-  <si>
-    <t>PL_LNG</t>
-  </si>
-  <si>
-    <t>PT_LNG</t>
-  </si>
-  <si>
-    <t>ES_LNG</t>
-  </si>
-  <si>
-    <t>TR_LNG</t>
-  </si>
-  <si>
-    <t>UK_LNG</t>
-  </si>
-  <si>
-    <t>EE_LNG</t>
-  </si>
-  <si>
-    <t>FI_LNG</t>
-  </si>
-  <si>
-    <t>DE_LNG</t>
-  </si>
-  <si>
-    <t>IE_LNG</t>
-  </si>
-  <si>
-    <t>LV_LNG</t>
-  </si>
-  <si>
-    <t>QA_LNG</t>
-  </si>
-  <si>
     <t>capacity_new</t>
+  </si>
+  <si>
+    <t>USA_LNG_exp</t>
+  </si>
+  <si>
+    <t>QA_LNG_exp</t>
   </si>
 </sst>
 </file>
@@ -1703,10 +1652,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="D2">
         <v>999999</v>
@@ -1717,10 +1666,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>999999</v>
@@ -1731,10 +1680,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>999999</v>
@@ -1745,10 +1694,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>999999</v>
@@ -1759,10 +1708,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <v>999999</v>
@@ -1773,10 +1722,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="D7">
         <v>999999</v>
@@ -1787,10 +1736,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="D8">
         <v>999999</v>
@@ -1801,10 +1750,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="D9">
         <v>999999</v>
@@ -1815,10 +1764,10 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="D10">
         <v>999999</v>
@@ -1829,10 +1778,10 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="D11">
         <v>999999</v>
@@ -1843,10 +1792,10 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="D12">
         <v>999999</v>
@@ -1857,10 +1806,10 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="D13">
         <v>999999</v>
@@ -1871,10 +1820,10 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="D14">
         <v>999999</v>
@@ -1885,10 +1834,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="D15">
         <v>999999</v>
@@ -1899,10 +1848,10 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="D16">
         <v>999999</v>
@@ -1913,10 +1862,10 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="D17">
         <v>999999</v>
@@ -1927,10 +1876,10 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="D18">
         <v>999999</v>
@@ -2295,10 +2244,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="D2">
         <v>999999</v>
@@ -2309,10 +2258,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>999999</v>
@@ -2323,10 +2272,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>999999</v>
@@ -2337,10 +2286,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>999999</v>
@@ -2351,10 +2300,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <v>999999</v>
@@ -2365,10 +2314,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="D7">
         <v>999999</v>
@@ -2379,10 +2328,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="D8">
         <v>999999</v>
@@ -2393,10 +2342,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="D9">
         <v>999999</v>
@@ -2407,10 +2356,10 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="D10">
         <v>999999</v>
@@ -2421,10 +2370,10 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="D11">
         <v>999999</v>
@@ -2435,10 +2384,10 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="D12">
         <v>999999</v>
@@ -2449,10 +2398,10 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="D13">
         <v>999999</v>
@@ -2463,10 +2412,10 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="D14">
         <v>999999</v>
@@ -2477,10 +2426,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="D15">
         <v>999999</v>
@@ -2491,10 +2440,10 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="D16">
         <v>999999</v>
@@ -2505,10 +2454,10 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="D17">
         <v>999999</v>
@@ -2519,10 +2468,10 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="D18">
         <v>999999</v>
@@ -2883,7 +2832,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
add 2024 including imports from RU to TR
input files and raw results
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/Szenarios_update_information.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE41426D-03F5-4EC5-93E5-396CA3AA20BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226603F8-5F58-4A18-B072-0B964A16121C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
     <sheet name="2024" sheetId="2" r:id="rId2"/>
-    <sheet name="2035" sheetId="7" r:id="rId3"/>
-    <sheet name="2024_USA" sheetId="3" r:id="rId4"/>
-    <sheet name="2024_QA" sheetId="4" r:id="rId5"/>
-    <sheet name="2024_NOR" sheetId="6" r:id="rId6"/>
-    <sheet name="2024_InvesPipes" sheetId="5" r:id="rId7"/>
+    <sheet name="2024_RU" sheetId="8" r:id="rId3"/>
+    <sheet name="2035" sheetId="7" r:id="rId4"/>
+    <sheet name="2024_USA" sheetId="3" r:id="rId5"/>
+    <sheet name="2024_QA" sheetId="4" r:id="rId6"/>
+    <sheet name="2024_NOR" sheetId="6" r:id="rId7"/>
+    <sheet name="2024_InvesPipes" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="64">
   <si>
     <t>Commodity</t>
   </si>
@@ -315,6 +316,19 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{5FC43969-1B01-492D-8BE5-75E3821DED5F}" name="Table138" displayName="Table138" ref="A1:D22" totalsRowShown="0">
+  <autoFilter ref="A1:D22" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{2DAE9C0A-78C3-4EFA-8359-B4F2B2094723}" name="Commodity"/>
+    <tableColumn id="2" xr3:uid="{1DB3EB9F-E32E-414B-91DF-2FF394BA75FD}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{26397183-6F02-4613-AABD-1612A731C03C}" name="Destination"/>
+    <tableColumn id="4" xr3:uid="{038DD090-2D84-464B-8512-1A59EB103458}" name="costs_new"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2E4244DF-E5BF-4A0E-8F99-4EC8DA9D37A0}" name="Table137" displayName="Table137" ref="A1:D24" totalsRowShown="0">
   <autoFilter ref="A1:D24" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
   <tableColumns count="4">
@@ -327,7 +341,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}" name="Table4" displayName="Table4" ref="A1:D41" totalsRowShown="0">
   <autoFilter ref="A1:D41" xr:uid="{6C9B7B4E-0449-486C-9164-35200836C20F}"/>
   <tableColumns count="4">
@@ -340,7 +354,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}" name="Table3" displayName="Table3" ref="A1:D41" totalsRowShown="0">
   <autoFilter ref="A1:D41" xr:uid="{E7B2FD70-7014-4EF2-BBAF-254111C22FD0}"/>
   <tableColumns count="4">
@@ -353,7 +367,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{FEB0F6EA-E60A-4566-BA0E-BF2AF5C97F48}" name="Table136" displayName="Table136" ref="A1:E28" totalsRowShown="0">
   <autoFilter ref="A1:E28" xr:uid="{77C8ED8C-002C-483F-834D-0100691BEA70}"/>
   <tableColumns count="5">
@@ -1269,6 +1283,333 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A81D7E-3F0C-4300-8157-D122A142A646}">
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22">
+        <v>999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{943B3CE1-E7F7-4C15-AD65-81C37CD6AF52}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1623,7 +1964,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8977CDA9-B827-4B14-B0EF-E8B18335E1FD}">
   <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2215,7 +2556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E7BF925-CC6B-405E-A306-8078742D0F1F}">
   <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2807,7 +3148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C547CAD-73AE-429A-84D2-4495A6C1A811}">
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3302,7 +3643,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23A2BBDA-BF95-4C19-8BF8-08ECCB4DC5E7}">
   <dimension ref="A1:E104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>